<commit_message>
Arreglado la frontera eficiente
</commit_message>
<xml_diff>
--- a/src/frontera_eficiente.xlsx
+++ b/src/frontera_eficiente.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E21"/>
+  <dimension ref="A1:E43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -445,342 +445,716 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>0.09320000000000001</v>
+        <v>0.07920000000000001</v>
       </c>
       <c r="B2" t="n">
-        <v>0.018509</v>
+        <v>0.031862</v>
       </c>
       <c r="C2" t="n">
-        <v>0.009299999999999999</v>
+        <v>0.0484</v>
       </c>
       <c r="D2" t="n">
-        <v>0.0372</v>
+        <v>0.0003</v>
       </c>
       <c r="E2" t="n">
-        <v>0.9535</v>
+        <v>0.9514</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>0.09520000000000001</v>
+        <v>0.08119999999999999</v>
       </c>
       <c r="B3" t="n">
-        <v>0.017558</v>
+        <v>0.028979</v>
       </c>
       <c r="C3" t="n">
-        <v>0.0343</v>
+        <v>0.09710000000000001</v>
       </c>
       <c r="D3" t="n">
-        <v>0.0621</v>
+        <v>0.0003</v>
       </c>
       <c r="E3" t="n">
-        <v>0.9035</v>
+        <v>0.9026</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>0.09719999999999999</v>
+        <v>0.0832</v>
       </c>
       <c r="B4" t="n">
-        <v>0.016657</v>
+        <v>0.026426</v>
       </c>
       <c r="C4" t="n">
-        <v>0.0629</v>
+        <v>0.1457</v>
       </c>
       <c r="D4" t="n">
-        <v>0.0835</v>
+        <v>0.0005</v>
       </c>
       <c r="E4" t="n">
-        <v>0.8536</v>
+        <v>0.8538</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>0.0992</v>
+        <v>0.0852</v>
       </c>
       <c r="B5" t="n">
-        <v>0.015856</v>
+        <v>0.024204</v>
       </c>
       <c r="C5" t="n">
-        <v>0.0851</v>
+        <v>0.1942</v>
       </c>
       <c r="D5" t="n">
-        <v>0.1112</v>
+        <v>0.0007</v>
       </c>
       <c r="E5" t="n">
-        <v>0.8037</v>
+        <v>0.8052</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>0.1012</v>
+        <v>0.0872</v>
       </c>
       <c r="B6" t="n">
-        <v>0.015105</v>
+        <v>0.022312</v>
       </c>
       <c r="C6" t="n">
-        <v>0.1108</v>
+        <v>0.2421</v>
       </c>
       <c r="D6" t="n">
-        <v>0.1354</v>
+        <v>0.0011</v>
       </c>
       <c r="E6" t="n">
-        <v>0.7538</v>
+        <v>0.7568</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>0.1032</v>
+        <v>0.0892</v>
       </c>
       <c r="B7" t="n">
-        <v>0.014404</v>
+        <v>0.020751</v>
       </c>
       <c r="C7" t="n">
-        <v>0.1414</v>
+        <v>0.2883</v>
       </c>
       <c r="D7" t="n">
-        <v>0.1548</v>
+        <v>0.0024</v>
       </c>
       <c r="E7" t="n">
-        <v>0.7038</v>
+        <v>0.7093</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>0.1052</v>
+        <v>0.0912</v>
       </c>
       <c r="B8" t="n">
-        <v>0.013804</v>
+        <v>0.019489</v>
       </c>
       <c r="C8" t="n">
-        <v>0.1635</v>
+        <v>0.3375</v>
       </c>
       <c r="D8" t="n">
-        <v>0.1826</v>
+        <v>0.0023</v>
       </c>
       <c r="E8" t="n">
-        <v>0.6539</v>
+        <v>0.6602</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>0.1072</v>
+        <v>0.09320000000000001</v>
       </c>
       <c r="B9" t="n">
-        <v>0.013253</v>
+        <v>0.018468</v>
       </c>
       <c r="C9" t="n">
-        <v>0.1907</v>
+        <v>0.3472</v>
       </c>
       <c r="D9" t="n">
-        <v>0.2053</v>
+        <v>0.0212</v>
       </c>
       <c r="E9" t="n">
-        <v>0.604</v>
+        <v>0.6316000000000001</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>0.1092</v>
+        <v>0.09520000000000001</v>
       </c>
       <c r="B10" t="n">
-        <v>0.012803</v>
+        <v>0.017538</v>
       </c>
       <c r="C10" t="n">
-        <v>0.2101</v>
+        <v>0.3606</v>
       </c>
       <c r="D10" t="n">
-        <v>0.2359</v>
+        <v>0.0383</v>
       </c>
       <c r="E10" t="n">
-        <v>0.554</v>
+        <v>0.6011</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>0.1112</v>
+        <v>0.09719999999999999</v>
       </c>
       <c r="B11" t="n">
-        <v>0.012402</v>
+        <v>0.016637</v>
       </c>
       <c r="C11" t="n">
-        <v>0.234</v>
+        <v>0.3439</v>
       </c>
       <c r="D11" t="n">
-        <v>0.2619</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="E11" t="n">
-        <v>0.5041</v>
+        <v>0.5861</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>0.1132</v>
+        <v>0.0992</v>
       </c>
       <c r="B12" t="n">
-        <v>0.012052</v>
+        <v>0.015826</v>
       </c>
       <c r="C12" t="n">
-        <v>0.2611</v>
+        <v>0.3454</v>
       </c>
       <c r="D12" t="n">
-        <v>0.2847</v>
+        <v>0.0929</v>
       </c>
       <c r="E12" t="n">
-        <v>0.4542</v>
+        <v>0.5617</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>0.1152</v>
+        <v>0.1012</v>
       </c>
       <c r="B13" t="n">
-        <v>0.011802</v>
+        <v>0.015075</v>
       </c>
       <c r="C13" t="n">
-        <v>0.2826</v>
+        <v>0.3373</v>
       </c>
       <c r="D13" t="n">
-        <v>0.3132</v>
+        <v>0.1204</v>
       </c>
       <c r="E13" t="n">
-        <v>0.4043</v>
+        <v>0.5423</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>0.1172</v>
+        <v>0.1032</v>
       </c>
       <c r="B14" t="n">
-        <v>0.011552</v>
+        <v>0.014414</v>
       </c>
       <c r="C14" t="n">
-        <v>0.3204</v>
+        <v>0.3487</v>
       </c>
       <c r="D14" t="n">
-        <v>0.3252</v>
+        <v>0.1385</v>
       </c>
       <c r="E14" t="n">
-        <v>0.3543</v>
+        <v>0.5128</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>0.1192</v>
+        <v>0.1052</v>
       </c>
       <c r="B15" t="n">
-        <v>0.011451</v>
+        <v>0.013814</v>
       </c>
       <c r="C15" t="n">
-        <v>0.3348</v>
+        <v>0.3504</v>
       </c>
       <c r="D15" t="n">
-        <v>0.3608</v>
+        <v>0.1612</v>
       </c>
       <c r="E15" t="n">
-        <v>0.3044</v>
+        <v>0.4884</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>0.1212</v>
+        <v>0.1072</v>
       </c>
       <c r="B16" t="n">
-        <v>0.011351</v>
+        <v>0.013243</v>
       </c>
       <c r="C16" t="n">
-        <v>0.37</v>
+        <v>0.3278</v>
       </c>
       <c r="D16" t="n">
-        <v>0.3755</v>
+        <v>0.1957</v>
       </c>
       <c r="E16" t="n">
-        <v>0.2545</v>
+        <v>0.4765</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>0.1232</v>
+        <v>0.1092</v>
       </c>
       <c r="B17" t="n">
-        <v>0.011401</v>
+        <v>0.012793</v>
       </c>
       <c r="C17" t="n">
-        <v>0.3823</v>
+        <v>0.3429</v>
       </c>
       <c r="D17" t="n">
-        <v>0.4131</v>
+        <v>0.2121</v>
       </c>
       <c r="E17" t="n">
-        <v>0.2046</v>
+        <v>0.4451</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>0.1252</v>
+        <v>0.1112</v>
       </c>
       <c r="B18" t="n">
-        <v>0.011451</v>
+        <v>0.012372</v>
       </c>
       <c r="C18" t="n">
-        <v>0.4107</v>
+        <v>0.3324</v>
       </c>
       <c r="D18" t="n">
-        <v>0.4347</v>
+        <v>0.2407</v>
       </c>
       <c r="E18" t="n">
-        <v>0.1546</v>
+        <v>0.4269</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>0.1272</v>
+        <v>0.1132</v>
       </c>
       <c r="B19" t="n">
-        <v>0.011602</v>
+        <v>0.012042</v>
       </c>
       <c r="C19" t="n">
-        <v>0.4334</v>
+        <v>0.3343</v>
       </c>
       <c r="D19" t="n">
-        <v>0.4619</v>
+        <v>0.2634</v>
       </c>
       <c r="E19" t="n">
-        <v>0.1047</v>
+        <v>0.4023</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>0.1292</v>
+        <v>0.1152</v>
       </c>
       <c r="B20" t="n">
-        <v>0.011802</v>
+        <v>0.011772</v>
       </c>
       <c r="C20" t="n">
-        <v>0.4594</v>
+        <v>0.3315</v>
       </c>
       <c r="D20" t="n">
-        <v>0.4859</v>
+        <v>0.2883</v>
       </c>
       <c r="E20" t="n">
-        <v>0.0548</v>
+        <v>0.3802</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
+        <v>0.1172</v>
+      </c>
+      <c r="B21" t="n">
+        <v>0.011562</v>
+      </c>
+      <c r="C21" t="n">
+        <v>0.324</v>
+      </c>
+      <c r="D21" t="n">
+        <v>0.3155</v>
+      </c>
+      <c r="E21" t="n">
+        <v>0.3604</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>0.1192</v>
+      </c>
+      <c r="B22" t="n">
+        <v>0.011441</v>
+      </c>
+      <c r="C22" t="n">
+        <v>0.3288</v>
+      </c>
+      <c r="D22" t="n">
+        <v>0.3368</v>
+      </c>
+      <c r="E22" t="n">
+        <v>0.3344</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>0.1212</v>
+      </c>
+      <c r="B23" t="n">
+        <v>0.011351</v>
+      </c>
+      <c r="C23" t="n">
+        <v>0.3088</v>
+      </c>
+      <c r="D23" t="n">
+        <v>0.37</v>
+      </c>
+      <c r="E23" t="n">
+        <v>0.3211</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>0.1232</v>
+      </c>
+      <c r="B24" t="n">
+        <v>0.011381</v>
+      </c>
+      <c r="C24" t="n">
+        <v>0.3251</v>
+      </c>
+      <c r="D24" t="n">
+        <v>0.3858</v>
+      </c>
+      <c r="E24" t="n">
+        <v>0.2891</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>0.1252</v>
+      </c>
+      <c r="B25" t="n">
+        <v>0.011441</v>
+      </c>
+      <c r="C25" t="n">
+        <v>0.3178</v>
+      </c>
+      <c r="D25" t="n">
+        <v>0.4129</v>
+      </c>
+      <c r="E25" t="n">
+        <v>0.2693</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>0.1272</v>
+      </c>
+      <c r="B26" t="n">
+        <v>0.011562</v>
+      </c>
+      <c r="C26" t="n">
+        <v>0.3018</v>
+      </c>
+      <c r="D26" t="n">
+        <v>0.4442</v>
+      </c>
+      <c r="E26" t="n">
+        <v>0.254</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>0.1292</v>
+      </c>
+      <c r="B27" t="n">
+        <v>0.011772</v>
+      </c>
+      <c r="C27" t="n">
+        <v>0.3037</v>
+      </c>
+      <c r="D27" t="n">
+        <v>0.4669</v>
+      </c>
+      <c r="E27" t="n">
+        <v>0.2294</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
         <v>0.1312</v>
       </c>
-      <c r="B21" t="n">
-        <v>0.012052</v>
-      </c>
-      <c r="C21" t="n">
-        <v>0.4896</v>
-      </c>
-      <c r="D21" t="n">
-        <v>0.5054999999999999</v>
-      </c>
-      <c r="E21" t="n">
-        <v>0.0048</v>
+      <c r="B28" t="n">
+        <v>0.012042</v>
+      </c>
+      <c r="C28" t="n">
+        <v>0.2972</v>
+      </c>
+      <c r="D28" t="n">
+        <v>0.4936</v>
+      </c>
+      <c r="E28" t="n">
+        <v>0.2092</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>0.1332</v>
+      </c>
+      <c r="B29" t="n">
+        <v>0.012402</v>
+      </c>
+      <c r="C29" t="n">
+        <v>0.3073</v>
+      </c>
+      <c r="D29" t="n">
+        <v>0.5124</v>
+      </c>
+      <c r="E29" t="n">
+        <v>0.1804</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>0.1352</v>
+      </c>
+      <c r="B30" t="n">
+        <v>0.012793</v>
+      </c>
+      <c r="C30" t="n">
+        <v>0.2901</v>
+      </c>
+      <c r="D30" t="n">
+        <v>0.5442</v>
+      </c>
+      <c r="E30" t="n">
+        <v>0.1656</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>0.1372</v>
+      </c>
+      <c r="B31" t="n">
+        <v>0.013273</v>
+      </c>
+      <c r="C31" t="n">
+        <v>0.2905</v>
+      </c>
+      <c r="D31" t="n">
+        <v>0.5677</v>
+      </c>
+      <c r="E31" t="n">
+        <v>0.1419</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>0.1392</v>
+      </c>
+      <c r="B32" t="n">
+        <v>0.013844</v>
+      </c>
+      <c r="C32" t="n">
+        <v>0.3022</v>
+      </c>
+      <c r="D32" t="n">
+        <v>0.5856</v>
+      </c>
+      <c r="E32" t="n">
+        <v>0.1122</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>0.1412</v>
+      </c>
+      <c r="B33" t="n">
+        <v>0.014444</v>
+      </c>
+      <c r="C33" t="n">
+        <v>0.293</v>
+      </c>
+      <c r="D33" t="n">
+        <v>0.6136</v>
+      </c>
+      <c r="E33" t="n">
+        <v>0.0934</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>0.1432</v>
+      </c>
+      <c r="B34" t="n">
+        <v>0.015135</v>
+      </c>
+      <c r="C34" t="n">
+        <v>0.2945</v>
+      </c>
+      <c r="D34" t="n">
+        <v>0.6365</v>
+      </c>
+      <c r="E34" t="n">
+        <v>0.06900000000000001</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>0.1452</v>
+      </c>
+      <c r="B35" t="n">
+        <v>0.015886</v>
+      </c>
+      <c r="C35" t="n">
+        <v>0.292</v>
+      </c>
+      <c r="D35" t="n">
+        <v>0.6613</v>
+      </c>
+      <c r="E35" t="n">
+        <v>0.0467</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>0.1472</v>
+      </c>
+      <c r="B36" t="n">
+        <v>0.016697</v>
+      </c>
+      <c r="C36" t="n">
+        <v>0.2857</v>
+      </c>
+      <c r="D36" t="n">
+        <v>0.6879</v>
+      </c>
+      <c r="E36" t="n">
+        <v>0.0264</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>0.1492</v>
+      </c>
+      <c r="B37" t="n">
+        <v>0.017568</v>
+      </c>
+      <c r="C37" t="n">
+        <v>0.2716</v>
+      </c>
+      <c r="D37" t="n">
+        <v>0.7183</v>
+      </c>
+      <c r="E37" t="n">
+        <v>0.0101</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="n">
+        <v>0.1512</v>
+      </c>
+      <c r="B38" t="n">
+        <v>0.018559</v>
+      </c>
+      <c r="C38" t="n">
+        <v>0.232</v>
+      </c>
+      <c r="D38" t="n">
+        <v>0.7611</v>
+      </c>
+      <c r="E38" t="n">
+        <v>0.007</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="n">
+        <v>0.1532</v>
+      </c>
+      <c r="B39" t="n">
+        <v>0.01973</v>
+      </c>
+      <c r="C39" t="n">
+        <v>0.1956</v>
+      </c>
+      <c r="D39" t="n">
+        <v>0.8022</v>
+      </c>
+      <c r="E39" t="n">
+        <v>0.0022</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="n">
+        <v>0.1552</v>
+      </c>
+      <c r="B40" t="n">
+        <v>0.021141</v>
+      </c>
+      <c r="C40" t="n">
+        <v>0.1528</v>
+      </c>
+      <c r="D40" t="n">
+        <v>0.8465</v>
+      </c>
+      <c r="E40" t="n">
+        <v>0.0008</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>0.1572</v>
+      </c>
+      <c r="B41" t="n">
+        <v>0.022823</v>
+      </c>
+      <c r="C41" t="n">
+        <v>0.1067</v>
+      </c>
+      <c r="D41" t="n">
+        <v>0.8923</v>
+      </c>
+      <c r="E41" t="n">
+        <v>0.001</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="n">
+        <v>0.1592</v>
+      </c>
+      <c r="B42" t="n">
+        <v>0.024715</v>
+      </c>
+      <c r="C42" t="n">
+        <v>0.06279999999999999</v>
+      </c>
+      <c r="D42" t="n">
+        <v>0.9370000000000001</v>
+      </c>
+      <c r="E42" t="n">
+        <v>0.0001</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="n">
+        <v>0.1612</v>
+      </c>
+      <c r="B43" t="n">
+        <v>0.026877</v>
+      </c>
+      <c r="C43" t="n">
+        <v>0.0173</v>
+      </c>
+      <c r="D43" t="n">
+        <v>0.9826</v>
+      </c>
+      <c r="E43" t="n">
+        <v>0.0001</v>
       </c>
     </row>
   </sheetData>

</xml_diff>